<commit_message>
demo: updated some forms
</commit_message>
<xml_diff>
--- a/Demo/ONCHO/epi/demo_oncho_epi_9999_1_site.xlsx
+++ b/Demo/ONCHO/epi/demo_oncho_epi_9999_1_site.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yumbad\Repositories\dsa-forms\Demo\ONCHO\epi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7120D581-7DBF-419C-A77F-002C62818C38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A11E05B-1D5B-4C5E-BF5D-02EEF60B4037}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="survey" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="569" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="202">
   <si>
     <t>type</t>
   </si>
@@ -643,6 +643,9 @@
   </si>
   <si>
     <t>${c_admin1}</t>
+  </si>
+  <si>
+    <t>${c_gps_type} = 'Manual Entry'</t>
   </si>
 </sst>
 </file>
@@ -1948,7 +1951,9 @@
       <c r="E27" s="23"/>
       <c r="F27" s="23"/>
       <c r="G27" s="23"/>
-      <c r="H27" s="23"/>
+      <c r="H27" s="23" t="s">
+        <v>166</v>
+      </c>
       <c r="I27" s="23"/>
       <c r="J27" s="18" t="s">
         <v>15</v>
@@ -1980,7 +1985,7 @@
         <v>173</v>
       </c>
       <c r="H28" s="23" t="s">
-        <v>166</v>
+        <v>201</v>
       </c>
       <c r="I28" s="23"/>
       <c r="J28" s="18" t="s">
@@ -2012,7 +2017,9 @@
       <c r="G29" s="23" t="s">
         <v>175</v>
       </c>
-      <c r="H29" s="23"/>
+      <c r="H29" s="23" t="s">
+        <v>201</v>
+      </c>
       <c r="I29" s="23"/>
       <c r="J29" s="18" t="s">
         <v>15</v>

</xml_diff>